<commit_message>
add support for excel export for player brackets of all sizes
</commit_message>
<xml_diff>
--- a/client/public/templates/bracket_players/12-player.xlsx
+++ b/client/public/templates/bracket_players/12-player.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bellahuang/Downloads/Players/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B18CC3F4-261A-3143-8AD1-10D164EA854D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04E3D13A-0017-4440-8464-2DEBB10F21C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="220" yWindow="780" windowWidth="34200" windowHeight="21360" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Poster" sheetId="1" r:id="rId1"/>
-    <sheet name="Booklet (left)" sheetId="2" r:id="rId2"/>
-    <sheet name="Booklet (right)" sheetId="3" r:id="rId3"/>
+    <sheet name="Full" sheetId="1" r:id="rId1"/>
+    <sheet name="Left" sheetId="2" r:id="rId2"/>
+    <sheet name="Right" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -398,80 +398,80 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -911,8 +911,8 @@
       <c r="Z3" s="5"/>
     </row>
     <row r="4" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A4" s="68"/>
-      <c r="B4" s="71"/>
+      <c r="A4" s="64"/>
+      <c r="B4" s="66"/>
       <c r="C4" s="6"/>
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
@@ -935,8 +935,8 @@
       <c r="Z4" s="5"/>
     </row>
     <row r="5" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A5" s="67"/>
-      <c r="B5" s="63"/>
+      <c r="A5" s="65"/>
+      <c r="B5" s="67"/>
       <c r="C5" s="7"/>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -963,14 +963,14 @@
       <c r="Z5" s="5"/>
     </row>
     <row r="6" spans="1:26" ht="16">
-      <c r="A6" s="70"/>
-      <c r="B6" s="65"/>
-      <c r="C6" s="72">
+      <c r="A6" s="62"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="68">
         <v>1</v>
       </c>
       <c r="D6" s="8"/>
-      <c r="E6" s="68"/>
-      <c r="F6" s="71"/>
+      <c r="E6" s="64"/>
+      <c r="F6" s="66"/>
       <c r="G6" s="4"/>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
@@ -995,10 +995,10 @@
     <row r="7" spans="1:26" ht="15.75" customHeight="1">
       <c r="A7" s="6"/>
       <c r="B7" s="9"/>
-      <c r="C7" s="73"/>
+      <c r="C7" s="69"/>
       <c r="D7" s="11"/>
-      <c r="E7" s="67"/>
-      <c r="F7" s="63"/>
+      <c r="E7" s="65"/>
+      <c r="F7" s="67"/>
       <c r="G7" s="12"/>
       <c r="H7" s="13"/>
       <c r="I7" s="5"/>
@@ -1017,18 +1017,18 @@
       <c r="Z7" s="5"/>
     </row>
     <row r="8" spans="1:26" ht="16">
-      <c r="A8" s="68"/>
-      <c r="B8" s="69"/>
+      <c r="A8" s="64"/>
+      <c r="B8" s="70"/>
       <c r="C8" s="14"/>
       <c r="D8" s="2"/>
-      <c r="E8" s="70"/>
-      <c r="F8" s="65"/>
-      <c r="G8" s="64">
+      <c r="E8" s="62"/>
+      <c r="F8" s="63"/>
+      <c r="G8" s="73">
         <v>5</v>
       </c>
       <c r="H8" s="15"/>
-      <c r="I8" s="68"/>
-      <c r="J8" s="71"/>
+      <c r="I8" s="64"/>
+      <c r="J8" s="66"/>
       <c r="K8" s="4"/>
       <c r="L8" s="5"/>
       <c r="M8" s="5"/>
@@ -1043,16 +1043,16 @@
       <c r="Z8" s="5"/>
     </row>
     <row r="9" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A9" s="67"/>
-      <c r="B9" s="63"/>
+      <c r="A9" s="65"/>
+      <c r="B9" s="67"/>
       <c r="C9" s="1"/>
       <c r="D9" s="5"/>
       <c r="E9" s="4"/>
       <c r="F9" s="5"/>
-      <c r="G9" s="65"/>
+      <c r="G9" s="63"/>
       <c r="H9" s="16"/>
-      <c r="I9" s="67"/>
-      <c r="J9" s="63"/>
+      <c r="I9" s="65"/>
+      <c r="J9" s="67"/>
       <c r="K9" s="17"/>
       <c r="L9" s="5"/>
       <c r="M9" s="5"/>
@@ -1071,12 +1071,12 @@
       <c r="Z9" s="5"/>
     </row>
     <row r="10" spans="1:26" ht="16">
-      <c r="A10" s="70"/>
-      <c r="B10" s="65"/>
+      <c r="A10" s="62"/>
+      <c r="B10" s="63"/>
       <c r="C10" s="4"/>
       <c r="D10" s="5"/>
-      <c r="E10" s="68"/>
-      <c r="F10" s="62"/>
+      <c r="E10" s="64"/>
+      <c r="F10" s="74"/>
       <c r="G10" s="18"/>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
@@ -1095,8 +1095,8 @@
     </row>
     <row r="11" spans="1:26" ht="15.75" customHeight="1">
       <c r="D11" s="2"/>
-      <c r="E11" s="67"/>
-      <c r="F11" s="63"/>
+      <c r="E11" s="65"/>
+      <c r="F11" s="67"/>
       <c r="G11" s="19"/>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
@@ -1118,8 +1118,8 @@
       <c r="B12" s="2"/>
       <c r="C12" s="1"/>
       <c r="D12" s="2"/>
-      <c r="E12" s="70"/>
-      <c r="F12" s="65"/>
+      <c r="E12" s="62"/>
+      <c r="F12" s="63"/>
       <c r="G12" s="4"/>
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
@@ -1145,12 +1145,12 @@
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
-      <c r="K13" s="64">
+      <c r="K13" s="73">
         <v>9</v>
       </c>
       <c r="L13" s="15"/>
-      <c r="M13" s="68"/>
-      <c r="N13" s="71"/>
+      <c r="M13" s="64"/>
+      <c r="N13" s="66"/>
       <c r="O13" s="5"/>
       <c r="P13" s="5"/>
       <c r="Q13" s="5"/>
@@ -1165,8 +1165,8 @@
       <c r="Z13" s="5"/>
     </row>
     <row r="14" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A14" s="68"/>
-      <c r="B14" s="71"/>
+      <c r="A14" s="64"/>
+      <c r="B14" s="66"/>
       <c r="C14" s="6"/>
       <c r="D14" s="2"/>
       <c r="E14" s="4"/>
@@ -1175,10 +1175,10 @@
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
-      <c r="K14" s="65"/>
+      <c r="K14" s="63"/>
       <c r="L14" s="16"/>
-      <c r="M14" s="67"/>
-      <c r="N14" s="63"/>
+      <c r="M14" s="65"/>
+      <c r="N14" s="67"/>
       <c r="O14" s="20"/>
       <c r="P14" s="13"/>
       <c r="Q14" s="5"/>
@@ -1193,8 +1193,8 @@
       <c r="Z14" s="5"/>
     </row>
     <row r="15" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A15" s="67"/>
-      <c r="B15" s="63"/>
+      <c r="A15" s="65"/>
+      <c r="B15" s="67"/>
       <c r="C15" s="7"/>
       <c r="D15" s="2"/>
       <c r="E15" s="4"/>
@@ -1218,14 +1218,14 @@
       <c r="Z15" s="5"/>
     </row>
     <row r="16" spans="1:26" ht="16">
-      <c r="A16" s="70"/>
-      <c r="B16" s="65"/>
-      <c r="C16" s="72">
+      <c r="A16" s="62"/>
+      <c r="B16" s="63"/>
+      <c r="C16" s="68">
         <v>2</v>
       </c>
       <c r="D16" s="8"/>
-      <c r="E16" s="68"/>
-      <c r="F16" s="71"/>
+      <c r="E16" s="64"/>
+      <c r="F16" s="66"/>
       <c r="G16" s="4"/>
       <c r="H16" s="5"/>
       <c r="I16" s="5"/>
@@ -1250,10 +1250,10 @@
     <row r="17" spans="1:26" ht="15.75" customHeight="1">
       <c r="A17" s="6"/>
       <c r="B17" s="9"/>
-      <c r="C17" s="73"/>
+      <c r="C17" s="69"/>
       <c r="D17" s="11"/>
-      <c r="E17" s="67"/>
-      <c r="F17" s="63"/>
+      <c r="E17" s="65"/>
+      <c r="F17" s="67"/>
       <c r="G17" s="12"/>
       <c r="H17" s="13"/>
       <c r="I17" s="5"/>
@@ -1276,18 +1276,18 @@
       <c r="Z17" s="5"/>
     </row>
     <row r="18" spans="1:26" ht="16">
-      <c r="A18" s="68"/>
-      <c r="B18" s="69"/>
+      <c r="A18" s="64"/>
+      <c r="B18" s="70"/>
       <c r="C18" s="14"/>
       <c r="D18" s="2"/>
-      <c r="E18" s="70"/>
-      <c r="F18" s="65"/>
-      <c r="G18" s="64">
+      <c r="E18" s="62"/>
+      <c r="F18" s="63"/>
+      <c r="G18" s="73">
         <v>6</v>
       </c>
       <c r="H18" s="15"/>
-      <c r="I18" s="66"/>
-      <c r="J18" s="62"/>
+      <c r="I18" s="75"/>
+      <c r="J18" s="74"/>
       <c r="K18" s="21"/>
       <c r="L18" s="13"/>
       <c r="M18" s="5"/>
@@ -1306,16 +1306,16 @@
       <c r="Z18" s="5"/>
     </row>
     <row r="19" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A19" s="67"/>
-      <c r="B19" s="63"/>
+      <c r="A19" s="65"/>
+      <c r="B19" s="67"/>
       <c r="C19" s="1"/>
       <c r="D19" s="2"/>
       <c r="E19" s="6"/>
       <c r="F19" s="9"/>
-      <c r="G19" s="65"/>
+      <c r="G19" s="63"/>
       <c r="H19" s="16"/>
-      <c r="I19" s="67"/>
-      <c r="J19" s="63"/>
+      <c r="I19" s="65"/>
+      <c r="J19" s="67"/>
       <c r="K19" s="4"/>
       <c r="L19" s="5"/>
       <c r="M19" s="5"/>
@@ -1334,12 +1334,12 @@
       <c r="Z19" s="5"/>
     </row>
     <row r="20" spans="1:26" ht="16">
-      <c r="A20" s="70"/>
-      <c r="B20" s="65"/>
+      <c r="A20" s="62"/>
+      <c r="B20" s="63"/>
       <c r="C20" s="4"/>
       <c r="D20" s="5"/>
-      <c r="E20" s="68"/>
-      <c r="F20" s="69"/>
+      <c r="E20" s="64"/>
+      <c r="F20" s="70"/>
       <c r="G20" s="22"/>
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
@@ -1366,8 +1366,8 @@
       <c r="B21" s="5"/>
       <c r="C21" s="4"/>
       <c r="D21" s="5"/>
-      <c r="E21" s="67"/>
-      <c r="F21" s="63"/>
+      <c r="E21" s="65"/>
+      <c r="F21" s="67"/>
       <c r="G21" s="12"/>
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
@@ -1394,8 +1394,8 @@
       <c r="B22" s="2"/>
       <c r="C22" s="1"/>
       <c r="D22" s="2"/>
-      <c r="E22" s="70"/>
-      <c r="F22" s="65"/>
+      <c r="E22" s="62"/>
+      <c r="F22" s="63"/>
       <c r="G22" s="4"/>
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
@@ -1429,12 +1429,12 @@
       <c r="L23" s="5"/>
       <c r="M23" s="5"/>
       <c r="N23" s="5"/>
-      <c r="O23" s="64">
+      <c r="O23" s="73">
         <v>11</v>
       </c>
       <c r="P23" s="15"/>
-      <c r="Q23" s="68"/>
-      <c r="R23" s="71"/>
+      <c r="Q23" s="64"/>
+      <c r="R23" s="66"/>
       <c r="S23" s="5"/>
       <c r="T23" s="5"/>
       <c r="U23" s="5"/>
@@ -1456,10 +1456,10 @@
       <c r="L24" s="5"/>
       <c r="M24" s="5"/>
       <c r="N24" s="5"/>
-      <c r="O24" s="65"/>
+      <c r="O24" s="63"/>
       <c r="P24" s="16"/>
-      <c r="Q24" s="67"/>
-      <c r="R24" s="63"/>
+      <c r="Q24" s="65"/>
+      <c r="R24" s="67"/>
       <c r="S24" s="5"/>
       <c r="T24" s="5"/>
       <c r="U24" s="5"/>
@@ -1470,8 +1470,8 @@
       <c r="Z24" s="5"/>
     </row>
     <row r="25" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A25" s="68"/>
-      <c r="B25" s="71"/>
+      <c r="A25" s="64"/>
+      <c r="B25" s="66"/>
       <c r="C25" s="6"/>
       <c r="D25" s="2"/>
       <c r="E25" s="4"/>
@@ -1495,8 +1495,8 @@
       <c r="Z25" s="5"/>
     </row>
     <row r="26" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A26" s="67"/>
-      <c r="B26" s="63"/>
+      <c r="A26" s="65"/>
+      <c r="B26" s="67"/>
       <c r="C26" s="7"/>
       <c r="D26" s="2"/>
       <c r="E26" s="4"/>
@@ -1523,14 +1523,14 @@
       <c r="Z26" s="5"/>
     </row>
     <row r="27" spans="1:26" ht="16">
-      <c r="A27" s="70"/>
-      <c r="B27" s="65"/>
-      <c r="C27" s="72">
+      <c r="A27" s="62"/>
+      <c r="B27" s="63"/>
+      <c r="C27" s="68">
         <v>3</v>
       </c>
       <c r="D27" s="8"/>
-      <c r="E27" s="68"/>
-      <c r="F27" s="71"/>
+      <c r="E27" s="64"/>
+      <c r="F27" s="66"/>
       <c r="G27" s="4"/>
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
@@ -1552,10 +1552,10 @@
     <row r="28" spans="1:26" ht="15.75" customHeight="1">
       <c r="A28" s="6"/>
       <c r="B28" s="9"/>
-      <c r="C28" s="73"/>
+      <c r="C28" s="69"/>
       <c r="D28" s="11"/>
-      <c r="E28" s="67"/>
-      <c r="F28" s="63"/>
+      <c r="E28" s="65"/>
+      <c r="F28" s="67"/>
       <c r="G28" s="12"/>
       <c r="H28" s="13"/>
       <c r="I28" s="5"/>
@@ -1575,18 +1575,18 @@
       <c r="Z28" s="5"/>
     </row>
     <row r="29" spans="1:26" ht="16">
-      <c r="A29" s="68"/>
-      <c r="B29" s="69"/>
+      <c r="A29" s="64"/>
+      <c r="B29" s="70"/>
       <c r="C29" s="14"/>
       <c r="D29" s="2"/>
-      <c r="E29" s="70"/>
-      <c r="F29" s="65"/>
-      <c r="G29" s="64">
+      <c r="E29" s="62"/>
+      <c r="F29" s="63"/>
+      <c r="G29" s="73">
         <v>7</v>
       </c>
       <c r="H29" s="15"/>
-      <c r="I29" s="66"/>
-      <c r="J29" s="62"/>
+      <c r="I29" s="75"/>
+      <c r="J29" s="74"/>
       <c r="K29" s="4"/>
       <c r="L29" s="5"/>
       <c r="M29" s="5"/>
@@ -1605,16 +1605,16 @@
       <c r="Z29" s="5"/>
     </row>
     <row r="30" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A30" s="67"/>
-      <c r="B30" s="63"/>
+      <c r="A30" s="65"/>
+      <c r="B30" s="67"/>
       <c r="C30" s="1"/>
       <c r="D30" s="2"/>
       <c r="E30" s="6"/>
       <c r="F30" s="9"/>
-      <c r="G30" s="65"/>
+      <c r="G30" s="63"/>
       <c r="H30" s="16"/>
-      <c r="I30" s="67"/>
-      <c r="J30" s="63"/>
+      <c r="I30" s="65"/>
+      <c r="J30" s="67"/>
       <c r="K30" s="17"/>
       <c r="L30" s="5"/>
       <c r="M30" s="5"/>
@@ -1631,12 +1631,12 @@
       <c r="Z30" s="5"/>
     </row>
     <row r="31" spans="1:26" ht="16">
-      <c r="A31" s="70"/>
-      <c r="B31" s="65"/>
+      <c r="A31" s="62"/>
+      <c r="B31" s="63"/>
       <c r="C31" s="4"/>
       <c r="D31" s="5"/>
-      <c r="E31" s="68"/>
-      <c r="F31" s="69"/>
+      <c r="E31" s="64"/>
+      <c r="F31" s="70"/>
       <c r="G31" s="10"/>
       <c r="K31" s="10"/>
       <c r="O31" s="5"/>
@@ -1655,8 +1655,8 @@
       <c r="B32" s="5"/>
       <c r="C32" s="4"/>
       <c r="D32" s="5"/>
-      <c r="E32" s="67"/>
-      <c r="F32" s="63"/>
+      <c r="E32" s="65"/>
+      <c r="F32" s="67"/>
       <c r="G32" s="12"/>
       <c r="K32" s="10"/>
       <c r="O32" s="5"/>
@@ -1677,8 +1677,8 @@
       <c r="B33" s="2"/>
       <c r="C33" s="1"/>
       <c r="D33" s="2"/>
-      <c r="E33" s="70"/>
-      <c r="F33" s="65"/>
+      <c r="E33" s="62"/>
+      <c r="F33" s="63"/>
       <c r="G33" s="4"/>
       <c r="H33" s="5"/>
       <c r="I33" s="5"/>
@@ -1698,8 +1698,8 @@
       <c r="Z33" s="5"/>
     </row>
     <row r="34" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A34" s="68"/>
-      <c r="B34" s="71"/>
+      <c r="A34" s="64"/>
+      <c r="B34" s="66"/>
       <c r="C34" s="6"/>
       <c r="D34" s="2"/>
       <c r="E34" s="4"/>
@@ -1707,12 +1707,12 @@
       <c r="H34" s="5"/>
       <c r="I34" s="5"/>
       <c r="J34" s="5"/>
-      <c r="K34" s="64">
+      <c r="K34" s="73">
         <v>10</v>
       </c>
       <c r="L34" s="15"/>
-      <c r="M34" s="66"/>
-      <c r="N34" s="62"/>
+      <c r="M34" s="75"/>
+      <c r="N34" s="74"/>
       <c r="O34" s="5"/>
       <c r="P34" s="13"/>
       <c r="Q34" s="5"/>
@@ -1727,17 +1727,17 @@
       <c r="Z34" s="5"/>
     </row>
     <row r="35" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A35" s="67"/>
-      <c r="B35" s="63"/>
+      <c r="A35" s="65"/>
+      <c r="B35" s="67"/>
       <c r="C35" s="7"/>
       <c r="D35" s="2"/>
       <c r="H35" s="5"/>
       <c r="I35" s="5"/>
       <c r="J35" s="5"/>
-      <c r="K35" s="65"/>
+      <c r="K35" s="63"/>
       <c r="L35" s="16"/>
-      <c r="M35" s="67"/>
-      <c r="N35" s="63"/>
+      <c r="M35" s="65"/>
+      <c r="N35" s="67"/>
       <c r="O35" s="20"/>
       <c r="Q35" s="5"/>
       <c r="R35" s="5"/>
@@ -1751,14 +1751,14 @@
       <c r="Z35" s="5"/>
     </row>
     <row r="36" spans="1:26" ht="16">
-      <c r="A36" s="70"/>
-      <c r="B36" s="65"/>
-      <c r="C36" s="72">
+      <c r="A36" s="62"/>
+      <c r="B36" s="63"/>
+      <c r="C36" s="68">
         <v>4</v>
       </c>
       <c r="D36" s="8"/>
-      <c r="E36" s="68"/>
-      <c r="F36" s="71"/>
+      <c r="E36" s="64"/>
+      <c r="F36" s="66"/>
       <c r="G36" s="4"/>
       <c r="H36" s="5"/>
       <c r="I36" s="5"/>
@@ -1778,10 +1778,10 @@
     <row r="37" spans="1:26" ht="15.75" customHeight="1">
       <c r="A37" s="6"/>
       <c r="B37" s="9"/>
-      <c r="C37" s="73"/>
+      <c r="C37" s="69"/>
       <c r="D37" s="11"/>
-      <c r="E37" s="67"/>
-      <c r="F37" s="63"/>
+      <c r="E37" s="65"/>
+      <c r="F37" s="67"/>
       <c r="G37" s="12"/>
       <c r="H37" s="13"/>
       <c r="I37" s="5"/>
@@ -1803,18 +1803,18 @@
       <c r="Z37" s="5"/>
     </row>
     <row r="38" spans="1:26" ht="16">
-      <c r="A38" s="68"/>
-      <c r="B38" s="69"/>
+      <c r="A38" s="64"/>
+      <c r="B38" s="70"/>
       <c r="C38" s="14"/>
       <c r="D38" s="2"/>
-      <c r="E38" s="70"/>
-      <c r="F38" s="65"/>
-      <c r="G38" s="64">
+      <c r="E38" s="62"/>
+      <c r="F38" s="63"/>
+      <c r="G38" s="73">
         <v>8</v>
       </c>
       <c r="H38" s="15"/>
-      <c r="I38" s="66"/>
-      <c r="J38" s="62"/>
+      <c r="I38" s="75"/>
+      <c r="J38" s="74"/>
       <c r="K38" s="18"/>
       <c r="L38" s="5"/>
       <c r="M38" s="5"/>
@@ -1833,16 +1833,16 @@
       <c r="Z38" s="5"/>
     </row>
     <row r="39" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A39" s="67"/>
-      <c r="B39" s="63"/>
+      <c r="A39" s="65"/>
+      <c r="B39" s="67"/>
       <c r="C39" s="1"/>
       <c r="D39" s="2"/>
       <c r="E39" s="6"/>
       <c r="F39" s="9"/>
-      <c r="G39" s="65"/>
+      <c r="G39" s="63"/>
       <c r="H39" s="16"/>
-      <c r="I39" s="67"/>
-      <c r="J39" s="63"/>
+      <c r="I39" s="65"/>
+      <c r="J39" s="67"/>
       <c r="L39" s="5"/>
       <c r="M39" s="5"/>
       <c r="N39" s="5"/>
@@ -1860,12 +1860,12 @@
       <c r="Z39" s="5"/>
     </row>
     <row r="40" spans="1:26" ht="16">
-      <c r="A40" s="70"/>
-      <c r="B40" s="65"/>
+      <c r="A40" s="62"/>
+      <c r="B40" s="63"/>
       <c r="C40" s="4"/>
       <c r="D40" s="5"/>
-      <c r="E40" s="68"/>
-      <c r="F40" s="69"/>
+      <c r="E40" s="64"/>
+      <c r="F40" s="70"/>
       <c r="G40" s="22"/>
       <c r="H40" s="13"/>
       <c r="I40" s="5"/>
@@ -1888,8 +1888,8 @@
       <c r="Z40" s="5"/>
     </row>
     <row r="41" spans="1:26" ht="15.75" customHeight="1">
-      <c r="E41" s="67"/>
-      <c r="F41" s="63"/>
+      <c r="E41" s="65"/>
+      <c r="F41" s="67"/>
       <c r="G41" s="12"/>
       <c r="H41" s="5"/>
       <c r="I41" s="5"/>
@@ -1912,8 +1912,8 @@
       <c r="Z41" s="5"/>
     </row>
     <row r="42" spans="1:26" ht="16">
-      <c r="E42" s="70"/>
-      <c r="F42" s="65"/>
+      <c r="E42" s="62"/>
+      <c r="F42" s="63"/>
       <c r="G42" s="4"/>
       <c r="H42" s="5"/>
       <c r="I42" s="5"/>
@@ -2035,8 +2035,8 @@
       <c r="Z48" s="5"/>
     </row>
     <row r="49" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A49" s="74"/>
-      <c r="B49" s="75"/>
+      <c r="A49" s="71"/>
+      <c r="B49" s="72"/>
       <c r="C49" s="1"/>
       <c r="D49" s="2"/>
       <c r="H49" s="5"/>
@@ -2060,8 +2060,8 @@
       <c r="Z49" s="5"/>
     </row>
     <row r="50" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A50" s="65"/>
-      <c r="B50" s="65"/>
+      <c r="A50" s="63"/>
+      <c r="B50" s="63"/>
       <c r="C50" s="1"/>
       <c r="D50" s="2"/>
       <c r="E50" s="4"/>
@@ -2138,8 +2138,8 @@
       <c r="Z52" s="5"/>
     </row>
     <row r="53" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A53" s="74"/>
-      <c r="B53" s="75"/>
+      <c r="A53" s="71"/>
+      <c r="B53" s="72"/>
       <c r="C53" s="1"/>
       <c r="D53" s="2"/>
       <c r="K53" s="4"/>
@@ -2160,8 +2160,8 @@
       <c r="Z53" s="5"/>
     </row>
     <row r="54" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A54" s="65"/>
-      <c r="B54" s="65"/>
+      <c r="A54" s="63"/>
+      <c r="B54" s="63"/>
       <c r="C54" s="1"/>
       <c r="D54" s="2"/>
       <c r="K54" s="4"/>
@@ -28691,37 +28691,40 @@
     </row>
   </sheetData>
   <mergeCells count="77">
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="E40:E41"/>
-    <mergeCell ref="F40:F41"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="F36:F37"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="N34:N35"/>
+    <mergeCell ref="G38:G39"/>
+    <mergeCell ref="I38:I39"/>
+    <mergeCell ref="J38:J39"/>
+    <mergeCell ref="G29:G30"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="K34:K35"/>
+    <mergeCell ref="M34:M35"/>
+    <mergeCell ref="J18:J19"/>
+    <mergeCell ref="O23:O24"/>
+    <mergeCell ref="Q23:Q24"/>
+    <mergeCell ref="R23:R24"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="I18:I19"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="B8:B9"/>
     <mergeCell ref="K13:K14"/>
     <mergeCell ref="M13:M14"/>
     <mergeCell ref="N13:N14"/>
@@ -28734,40 +28737,37 @@
     <mergeCell ref="G8:G9"/>
     <mergeCell ref="I8:I9"/>
     <mergeCell ref="J8:J9"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="F16:F17"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="G18:G19"/>
-    <mergeCell ref="I18:I19"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="J18:J19"/>
-    <mergeCell ref="O23:O24"/>
-    <mergeCell ref="Q23:Q24"/>
-    <mergeCell ref="R23:R24"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="N34:N35"/>
-    <mergeCell ref="G38:G39"/>
-    <mergeCell ref="I38:I39"/>
-    <mergeCell ref="J38:J39"/>
-    <mergeCell ref="G29:G30"/>
-    <mergeCell ref="I29:I30"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="K34:K35"/>
-    <mergeCell ref="M34:M35"/>
+    <mergeCell ref="F40:F41"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="E36:E37"/>
+    <mergeCell ref="F36:F37"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="E40:E41"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:C28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -28802,8 +28802,8 @@
       <c r="M1" s="5"/>
     </row>
     <row r="2" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A2" s="79"/>
-      <c r="B2" s="81"/>
+      <c r="A2" s="76"/>
+      <c r="B2" s="77"/>
       <c r="C2" s="25"/>
       <c r="D2" s="26"/>
       <c r="E2" s="23"/>
@@ -28817,8 +28817,8 @@
       <c r="M2" s="5"/>
     </row>
     <row r="3" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A3" s="67"/>
-      <c r="B3" s="63"/>
+      <c r="A3" s="65"/>
+      <c r="B3" s="67"/>
       <c r="C3" s="27"/>
       <c r="D3" s="26"/>
       <c r="E3" s="23"/>
@@ -28832,9 +28832,9 @@
       <c r="M3" s="5"/>
     </row>
     <row r="4" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A4" s="64"/>
-      <c r="B4" s="65"/>
-      <c r="C4" s="82">
+      <c r="A4" s="73"/>
+      <c r="B4" s="63"/>
+      <c r="C4" s="78">
         <v>1</v>
       </c>
       <c r="D4" s="25"/>
@@ -28851,7 +28851,7 @@
     <row r="5" spans="1:13" ht="15.75" customHeight="1">
       <c r="A5" s="28"/>
       <c r="B5" s="29"/>
-      <c r="C5" s="73"/>
+      <c r="C5" s="69"/>
       <c r="D5" s="27"/>
       <c r="E5" s="23"/>
       <c r="F5" s="24"/>
@@ -28864,8 +28864,8 @@
       <c r="M5" s="5"/>
     </row>
     <row r="6" spans="1:13" ht="16">
-      <c r="A6" s="83"/>
-      <c r="B6" s="84"/>
+      <c r="A6" s="82"/>
+      <c r="B6" s="79"/>
       <c r="C6" s="30"/>
       <c r="D6" s="27"/>
       <c r="E6" s="31"/>
@@ -28879,10 +28879,10 @@
       <c r="M6" s="5"/>
     </row>
     <row r="7" spans="1:13" ht="16">
-      <c r="A7" s="67"/>
-      <c r="B7" s="63"/>
+      <c r="A7" s="65"/>
+      <c r="B7" s="67"/>
       <c r="C7" s="26"/>
-      <c r="D7" s="82">
+      <c r="D7" s="78">
         <v>5</v>
       </c>
       <c r="E7" s="31"/>
@@ -28896,10 +28896,10 @@
       <c r="M7" s="5"/>
     </row>
     <row r="8" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A8" s="78"/>
-      <c r="B8" s="65"/>
+      <c r="A8" s="80"/>
+      <c r="B8" s="63"/>
       <c r="C8" s="26"/>
-      <c r="D8" s="73"/>
+      <c r="D8" s="69"/>
       <c r="E8" s="32"/>
       <c r="F8" s="24"/>
       <c r="G8" s="24"/>
@@ -28926,8 +28926,8 @@
       <c r="M9" s="5"/>
     </row>
     <row r="10" spans="1:13" ht="16">
-      <c r="A10" s="83"/>
-      <c r="B10" s="84"/>
+      <c r="A10" s="82"/>
+      <c r="B10" s="79"/>
       <c r="C10" s="25"/>
       <c r="D10" s="30"/>
       <c r="E10" s="33"/>
@@ -28941,8 +28941,8 @@
       <c r="M10" s="5"/>
     </row>
     <row r="11" spans="1:13" ht="16">
-      <c r="A11" s="67"/>
-      <c r="B11" s="63"/>
+      <c r="A11" s="65"/>
+      <c r="B11" s="67"/>
       <c r="C11" s="26"/>
       <c r="D11" s="26"/>
       <c r="E11" s="33"/>
@@ -28975,7 +28975,7 @@
       <c r="B13" s="2"/>
       <c r="C13" s="23"/>
       <c r="D13" s="23"/>
-      <c r="E13" s="76">
+      <c r="E13" s="81">
         <v>9</v>
       </c>
       <c r="G13" s="24"/>
@@ -28987,11 +28987,11 @@
       <c r="M13" s="5"/>
     </row>
     <row r="14" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A14" s="79"/>
-      <c r="B14" s="77"/>
+      <c r="A14" s="76"/>
+      <c r="B14" s="83"/>
       <c r="C14" s="36"/>
       <c r="D14" s="23"/>
-      <c r="E14" s="73"/>
+      <c r="E14" s="69"/>
       <c r="F14" s="35"/>
       <c r="G14" s="24"/>
       <c r="H14" s="24"/>
@@ -29002,8 +29002,8 @@
       <c r="M14" s="5"/>
     </row>
     <row r="15" spans="1:13" ht="16">
-      <c r="A15" s="67"/>
-      <c r="B15" s="63"/>
+      <c r="A15" s="65"/>
+      <c r="B15" s="67"/>
       <c r="C15" s="34"/>
       <c r="D15" s="23"/>
       <c r="E15" s="33"/>
@@ -29017,9 +29017,9 @@
       <c r="M15" s="5"/>
     </row>
     <row r="16" spans="1:13" ht="16">
-      <c r="A16" s="80"/>
-      <c r="B16" s="65"/>
-      <c r="C16" s="76">
+      <c r="A16" s="84"/>
+      <c r="B16" s="63"/>
+      <c r="C16" s="81">
         <v>2</v>
       </c>
       <c r="D16" s="36"/>
@@ -29036,7 +29036,7 @@
     <row r="17" spans="1:13" ht="16">
       <c r="A17" s="6"/>
       <c r="B17" s="9"/>
-      <c r="C17" s="73"/>
+      <c r="C17" s="69"/>
       <c r="D17" s="34"/>
       <c r="E17" s="33"/>
       <c r="F17" s="37"/>
@@ -29049,8 +29049,8 @@
       <c r="M17" s="5"/>
     </row>
     <row r="18" spans="1:13" ht="16">
-      <c r="A18" s="79"/>
-      <c r="B18" s="77"/>
+      <c r="A18" s="76"/>
+      <c r="B18" s="83"/>
       <c r="C18" s="38"/>
       <c r="D18" s="34"/>
       <c r="E18" s="33"/>
@@ -29064,10 +29064,10 @@
       <c r="M18" s="5"/>
     </row>
     <row r="19" spans="1:13" ht="16">
-      <c r="A19" s="67"/>
-      <c r="B19" s="63"/>
+      <c r="A19" s="65"/>
+      <c r="B19" s="67"/>
       <c r="C19" s="23"/>
-      <c r="D19" s="76">
+      <c r="D19" s="81">
         <v>6</v>
       </c>
       <c r="E19" s="39"/>
@@ -29081,10 +29081,10 @@
       <c r="M19" s="5"/>
     </row>
     <row r="20" spans="1:13" ht="16">
-      <c r="A20" s="78"/>
-      <c r="B20" s="65"/>
+      <c r="A20" s="80"/>
+      <c r="B20" s="63"/>
       <c r="C20" s="23"/>
-      <c r="D20" s="73"/>
+      <c r="D20" s="69"/>
       <c r="E20" s="31"/>
       <c r="F20" s="37"/>
       <c r="G20" s="24"/>
@@ -29111,8 +29111,8 @@
       <c r="M21" s="5"/>
     </row>
     <row r="22" spans="1:13" ht="16">
-      <c r="A22" s="79"/>
-      <c r="B22" s="77"/>
+      <c r="A22" s="76"/>
+      <c r="B22" s="83"/>
       <c r="C22" s="23"/>
       <c r="D22" s="38"/>
       <c r="E22" s="31"/>
@@ -29126,8 +29126,8 @@
       <c r="M22" s="5"/>
     </row>
     <row r="23" spans="1:13" ht="16">
-      <c r="A23" s="67"/>
-      <c r="B23" s="63"/>
+      <c r="A23" s="65"/>
+      <c r="B23" s="67"/>
       <c r="C23" s="43"/>
       <c r="D23" s="23"/>
       <c r="E23" s="31"/>
@@ -29146,7 +29146,7 @@
       <c r="C24" s="23"/>
       <c r="D24" s="23"/>
       <c r="E24" s="31"/>
-      <c r="F24" s="78">
+      <c r="F24" s="80">
         <v>11</v>
       </c>
       <c r="G24" s="45"/>
@@ -29163,7 +29163,7 @@
       <c r="C25" s="23"/>
       <c r="D25" s="23"/>
       <c r="E25" s="31"/>
-      <c r="F25" s="65"/>
+      <c r="F25" s="63"/>
       <c r="G25" s="44"/>
       <c r="H25" s="24"/>
       <c r="I25" s="5"/>
@@ -29173,8 +29173,8 @@
       <c r="M25" s="5"/>
     </row>
     <row r="26" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A26" s="79"/>
-      <c r="B26" s="81"/>
+      <c r="A26" s="76"/>
+      <c r="B26" s="77"/>
       <c r="C26" s="25"/>
       <c r="D26" s="26"/>
       <c r="E26" s="23"/>
@@ -29188,8 +29188,8 @@
       <c r="M26" s="5"/>
     </row>
     <row r="27" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A27" s="67"/>
-      <c r="B27" s="63"/>
+      <c r="A27" s="65"/>
+      <c r="B27" s="67"/>
       <c r="C27" s="27"/>
       <c r="D27" s="26"/>
       <c r="E27" s="23"/>
@@ -29203,9 +29203,9 @@
       <c r="M27" s="5"/>
     </row>
     <row r="28" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A28" s="64"/>
-      <c r="B28" s="65"/>
-      <c r="C28" s="82">
+      <c r="A28" s="73"/>
+      <c r="B28" s="63"/>
+      <c r="C28" s="78">
         <v>3</v>
       </c>
       <c r="D28" s="25"/>
@@ -29222,7 +29222,7 @@
     <row r="29" spans="1:13" ht="15.75" customHeight="1">
       <c r="A29" s="28"/>
       <c r="B29" s="29"/>
-      <c r="C29" s="73"/>
+      <c r="C29" s="69"/>
       <c r="D29" s="27"/>
       <c r="E29" s="23"/>
       <c r="F29" s="37"/>
@@ -29235,8 +29235,8 @@
       <c r="M29" s="5"/>
     </row>
     <row r="30" spans="1:13" ht="16">
-      <c r="A30" s="83"/>
-      <c r="B30" s="84"/>
+      <c r="A30" s="82"/>
+      <c r="B30" s="79"/>
       <c r="C30" s="30"/>
       <c r="D30" s="27"/>
       <c r="E30" s="31"/>
@@ -29250,10 +29250,10 @@
       <c r="M30" s="5"/>
     </row>
     <row r="31" spans="1:13" ht="16">
-      <c r="A31" s="67"/>
-      <c r="B31" s="63"/>
+      <c r="A31" s="65"/>
+      <c r="B31" s="67"/>
       <c r="C31" s="26"/>
-      <c r="D31" s="82">
+      <c r="D31" s="78">
         <v>7</v>
       </c>
       <c r="E31" s="31"/>
@@ -29267,10 +29267,10 @@
       <c r="M31" s="5"/>
     </row>
     <row r="32" spans="1:13" ht="16">
-      <c r="A32" s="78"/>
-      <c r="B32" s="65"/>
+      <c r="A32" s="80"/>
+      <c r="B32" s="63"/>
       <c r="C32" s="26"/>
-      <c r="D32" s="73"/>
+      <c r="D32" s="69"/>
       <c r="E32" s="46"/>
       <c r="F32" s="37"/>
       <c r="G32" s="24"/>
@@ -29297,8 +29297,8 @@
       <c r="M33" s="5"/>
     </row>
     <row r="34" spans="1:13" ht="16">
-      <c r="A34" s="83"/>
-      <c r="B34" s="84"/>
+      <c r="A34" s="82"/>
+      <c r="B34" s="79"/>
       <c r="C34" s="25"/>
       <c r="D34" s="30"/>
       <c r="E34" s="33"/>
@@ -29312,8 +29312,8 @@
       <c r="M34" s="5"/>
     </row>
     <row r="35" spans="1:13" ht="16">
-      <c r="A35" s="67"/>
-      <c r="B35" s="63"/>
+      <c r="A35" s="65"/>
+      <c r="B35" s="67"/>
       <c r="C35" s="26"/>
       <c r="D35" s="26"/>
       <c r="E35" s="33"/>
@@ -29346,7 +29346,7 @@
       <c r="B37" s="2"/>
       <c r="C37" s="23"/>
       <c r="D37" s="23"/>
-      <c r="E37" s="76">
+      <c r="E37" s="81">
         <v>10</v>
       </c>
       <c r="F37" s="47"/>
@@ -29359,11 +29359,11 @@
       <c r="M37" s="5"/>
     </row>
     <row r="38" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A38" s="79"/>
-      <c r="B38" s="77"/>
+      <c r="A38" s="76"/>
+      <c r="B38" s="83"/>
       <c r="C38" s="36"/>
       <c r="D38" s="23"/>
-      <c r="E38" s="73"/>
+      <c r="E38" s="69"/>
       <c r="F38" s="24"/>
       <c r="G38" s="24"/>
       <c r="H38" s="24"/>
@@ -29374,8 +29374,8 @@
       <c r="M38" s="5"/>
     </row>
     <row r="39" spans="1:13" ht="16">
-      <c r="A39" s="67"/>
-      <c r="B39" s="63"/>
+      <c r="A39" s="65"/>
+      <c r="B39" s="67"/>
       <c r="C39" s="34"/>
       <c r="D39" s="23"/>
       <c r="E39" s="33"/>
@@ -29389,9 +29389,9 @@
       <c r="M39" s="5"/>
     </row>
     <row r="40" spans="1:13" ht="16">
-      <c r="A40" s="80"/>
-      <c r="B40" s="65"/>
-      <c r="C40" s="76">
+      <c r="A40" s="84"/>
+      <c r="B40" s="63"/>
+      <c r="C40" s="81">
         <v>4</v>
       </c>
       <c r="D40" s="36"/>
@@ -29408,7 +29408,7 @@
     <row r="41" spans="1:13" ht="16">
       <c r="A41" s="6"/>
       <c r="B41" s="9"/>
-      <c r="C41" s="73"/>
+      <c r="C41" s="69"/>
       <c r="D41" s="34"/>
       <c r="E41" s="33"/>
       <c r="F41" s="24"/>
@@ -29421,8 +29421,8 @@
       <c r="M41" s="5"/>
     </row>
     <row r="42" spans="1:13" ht="16">
-      <c r="A42" s="79"/>
-      <c r="B42" s="77"/>
+      <c r="A42" s="76"/>
+      <c r="B42" s="83"/>
       <c r="C42" s="38"/>
       <c r="D42" s="34"/>
       <c r="E42" s="33"/>
@@ -29436,10 +29436,10 @@
       <c r="M42" s="5"/>
     </row>
     <row r="43" spans="1:13" ht="16">
-      <c r="A43" s="67"/>
-      <c r="B43" s="63"/>
+      <c r="A43" s="65"/>
+      <c r="B43" s="67"/>
       <c r="C43" s="23"/>
-      <c r="D43" s="76">
+      <c r="D43" s="81">
         <v>8</v>
       </c>
       <c r="E43" s="39"/>
@@ -29453,10 +29453,10 @@
       <c r="M43" s="5"/>
     </row>
     <row r="44" spans="1:13" ht="16">
-      <c r="A44" s="78"/>
-      <c r="B44" s="65"/>
+      <c r="A44" s="80"/>
+      <c r="B44" s="63"/>
       <c r="C44" s="23"/>
-      <c r="D44" s="73"/>
+      <c r="D44" s="69"/>
       <c r="E44" s="31"/>
       <c r="F44" s="24"/>
       <c r="G44" s="24"/>
@@ -29483,8 +29483,8 @@
       <c r="M45" s="5"/>
     </row>
     <row r="46" spans="1:13" ht="16">
-      <c r="A46" s="79"/>
-      <c r="B46" s="77"/>
+      <c r="A46" s="76"/>
+      <c r="B46" s="83"/>
       <c r="C46" s="23"/>
       <c r="D46" s="38"/>
       <c r="E46" s="31"/>
@@ -29498,8 +29498,8 @@
       <c r="M46" s="5"/>
     </row>
     <row r="47" spans="1:13" ht="16">
-      <c r="A47" s="67"/>
-      <c r="B47" s="63"/>
+      <c r="A47" s="65"/>
+      <c r="B47" s="67"/>
       <c r="C47" s="43"/>
       <c r="D47" s="23"/>
       <c r="E47" s="31"/>
@@ -43929,11 +43929,28 @@
     </row>
   </sheetData>
   <mergeCells count="43">
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="D43:D44"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A42:A43"/>
+    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="B34:B35"/>
     <mergeCell ref="D7:D8"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="D19:D20"/>
@@ -43950,28 +43967,11 @@
     <mergeCell ref="A18:A19"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="A22:A23"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="A46:A47"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="D43:D44"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A42:A43"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="B6:B7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -44011,8 +44011,8 @@
       <c r="C2" s="23"/>
       <c r="D2" s="26"/>
       <c r="E2" s="25"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="81"/>
+      <c r="F2" s="76"/>
+      <c r="G2" s="77"/>
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
@@ -44026,8 +44026,8 @@
       <c r="C3" s="23"/>
       <c r="D3" s="26"/>
       <c r="E3" s="48"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="63"/>
+      <c r="F3" s="65"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="5"/>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
@@ -44040,10 +44040,10 @@
       <c r="B4" s="24"/>
       <c r="C4" s="23"/>
       <c r="D4" s="26"/>
-      <c r="E4" s="91">
+      <c r="E4" s="85">
         <v>1</v>
       </c>
-      <c r="F4" s="92"/>
+      <c r="F4" s="87"/>
       <c r="G4" s="88"/>
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
@@ -44073,8 +44073,8 @@
       <c r="C6" s="31"/>
       <c r="D6" s="49"/>
       <c r="E6" s="51"/>
-      <c r="F6" s="83"/>
-      <c r="G6" s="84"/>
+      <c r="F6" s="82"/>
+      <c r="G6" s="79"/>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
@@ -44086,12 +44086,12 @@
       <c r="A7" s="24"/>
       <c r="B7" s="24"/>
       <c r="C7" s="31"/>
-      <c r="D7" s="91">
+      <c r="D7" s="85">
         <v>5</v>
       </c>
       <c r="E7" s="26"/>
-      <c r="F7" s="67"/>
-      <c r="G7" s="63"/>
+      <c r="F7" s="65"/>
+      <c r="G7" s="67"/>
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
       <c r="J7" s="5"/>
@@ -44105,8 +44105,8 @@
       <c r="C8" s="52"/>
       <c r="D8" s="86"/>
       <c r="E8" s="26"/>
-      <c r="F8" s="78"/>
-      <c r="G8" s="65"/>
+      <c r="F8" s="80"/>
+      <c r="G8" s="63"/>
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
@@ -44135,8 +44135,8 @@
       <c r="C10" s="53"/>
       <c r="D10" s="54"/>
       <c r="E10" s="25"/>
-      <c r="F10" s="83"/>
-      <c r="G10" s="84"/>
+      <c r="F10" s="82"/>
+      <c r="G10" s="79"/>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
@@ -44150,8 +44150,8 @@
       <c r="C11" s="53"/>
       <c r="D11" s="26"/>
       <c r="E11" s="26"/>
-      <c r="F11" s="67"/>
-      <c r="G11" s="63"/>
+      <c r="F11" s="65"/>
+      <c r="G11" s="67"/>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
       <c r="J11" s="5"/>
@@ -44177,7 +44177,7 @@
     <row r="13" spans="1:13" ht="15.75" customHeight="1">
       <c r="A13" s="24"/>
       <c r="B13" s="24"/>
-      <c r="C13" s="85">
+      <c r="C13" s="89">
         <v>9</v>
       </c>
       <c r="D13" s="23"/>
@@ -44197,8 +44197,8 @@
       <c r="C14" s="86"/>
       <c r="D14" s="23"/>
       <c r="E14" s="36"/>
-      <c r="F14" s="79"/>
-      <c r="G14" s="77"/>
+      <c r="F14" s="76"/>
+      <c r="G14" s="83"/>
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
@@ -44212,8 +44212,8 @@
       <c r="C15" s="53"/>
       <c r="D15" s="23"/>
       <c r="E15" s="57"/>
-      <c r="F15" s="67"/>
-      <c r="G15" s="63"/>
+      <c r="F15" s="65"/>
+      <c r="G15" s="67"/>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
@@ -44226,10 +44226,10 @@
       <c r="B16" s="44"/>
       <c r="C16" s="53"/>
       <c r="D16" s="23"/>
-      <c r="E16" s="85">
+      <c r="E16" s="89">
         <v>2</v>
       </c>
-      <c r="F16" s="87"/>
+      <c r="F16" s="90"/>
       <c r="G16" s="88"/>
       <c r="H16" s="5"/>
       <c r="I16" s="5"/>
@@ -44259,8 +44259,8 @@
       <c r="C18" s="53"/>
       <c r="D18" s="55"/>
       <c r="E18" s="59"/>
-      <c r="F18" s="90"/>
-      <c r="G18" s="89"/>
+      <c r="F18" s="91"/>
+      <c r="G18" s="92"/>
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
       <c r="J18" s="5"/>
@@ -44272,12 +44272,12 @@
       <c r="A19" s="37"/>
       <c r="B19" s="24"/>
       <c r="C19" s="60"/>
-      <c r="D19" s="85">
+      <c r="D19" s="89">
         <v>6</v>
       </c>
       <c r="E19" s="23"/>
-      <c r="F19" s="67"/>
-      <c r="G19" s="63"/>
+      <c r="F19" s="65"/>
+      <c r="G19" s="67"/>
       <c r="H19" s="5"/>
       <c r="I19" s="5"/>
       <c r="J19" s="5"/>
@@ -44291,8 +44291,8 @@
       <c r="C20" s="31"/>
       <c r="D20" s="86"/>
       <c r="E20" s="23"/>
-      <c r="F20" s="78"/>
-      <c r="G20" s="65"/>
+      <c r="F20" s="80"/>
+      <c r="G20" s="63"/>
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
@@ -44321,8 +44321,8 @@
       <c r="C22" s="31"/>
       <c r="D22" s="61"/>
       <c r="E22" s="23"/>
-      <c r="F22" s="79"/>
-      <c r="G22" s="77"/>
+      <c r="F22" s="76"/>
+      <c r="G22" s="83"/>
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
       <c r="J22" s="5"/>
@@ -44336,8 +44336,8 @@
       <c r="C23" s="31"/>
       <c r="D23" s="23"/>
       <c r="E23" s="43"/>
-      <c r="F23" s="67"/>
-      <c r="G23" s="63"/>
+      <c r="F23" s="65"/>
+      <c r="G23" s="67"/>
       <c r="H23" s="5"/>
       <c r="I23" s="5"/>
       <c r="J23" s="5"/>
@@ -44347,7 +44347,7 @@
     </row>
     <row r="24" spans="1:13" ht="16">
       <c r="A24" s="47"/>
-      <c r="B24" s="78">
+      <c r="B24" s="80">
         <v>11</v>
       </c>
       <c r="C24" s="31"/>
@@ -44364,7 +44364,7 @@
     </row>
     <row r="25" spans="1:13" ht="16">
       <c r="A25" s="37"/>
-      <c r="B25" s="65"/>
+      <c r="B25" s="63"/>
       <c r="C25" s="31"/>
       <c r="D25" s="23"/>
       <c r="E25" s="23"/>
@@ -44383,8 +44383,8 @@
       <c r="C26" s="23"/>
       <c r="D26" s="26"/>
       <c r="E26" s="25"/>
-      <c r="F26" s="79"/>
-      <c r="G26" s="81"/>
+      <c r="F26" s="76"/>
+      <c r="G26" s="77"/>
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
       <c r="J26" s="5"/>
@@ -44398,8 +44398,8 @@
       <c r="C27" s="23"/>
       <c r="D27" s="26"/>
       <c r="E27" s="48"/>
-      <c r="F27" s="67"/>
-      <c r="G27" s="63"/>
+      <c r="F27" s="65"/>
+      <c r="G27" s="67"/>
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
       <c r="J27" s="5"/>
@@ -44412,10 +44412,10 @@
       <c r="B28" s="23"/>
       <c r="C28" s="23"/>
       <c r="D28" s="26"/>
-      <c r="E28" s="91">
+      <c r="E28" s="85">
         <v>3</v>
       </c>
-      <c r="F28" s="92"/>
+      <c r="F28" s="87"/>
       <c r="G28" s="88"/>
       <c r="H28" s="5"/>
       <c r="I28" s="5"/>
@@ -44445,8 +44445,8 @@
       <c r="C30" s="31"/>
       <c r="D30" s="49"/>
       <c r="E30" s="51"/>
-      <c r="F30" s="83"/>
-      <c r="G30" s="84"/>
+      <c r="F30" s="82"/>
+      <c r="G30" s="79"/>
       <c r="H30" s="5"/>
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
@@ -44458,12 +44458,12 @@
       <c r="A31" s="37"/>
       <c r="B31" s="24"/>
       <c r="C31" s="31"/>
-      <c r="D31" s="91">
+      <c r="D31" s="85">
         <v>7</v>
       </c>
       <c r="E31" s="26"/>
-      <c r="F31" s="67"/>
-      <c r="G31" s="63"/>
+      <c r="F31" s="65"/>
+      <c r="G31" s="67"/>
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
       <c r="J31" s="5"/>
@@ -44477,8 +44477,8 @@
       <c r="C32" s="52"/>
       <c r="D32" s="86"/>
       <c r="E32" s="26"/>
-      <c r="F32" s="78"/>
-      <c r="G32" s="65"/>
+      <c r="F32" s="80"/>
+      <c r="G32" s="63"/>
       <c r="H32" s="5"/>
       <c r="I32" s="5"/>
       <c r="J32" s="5"/>
@@ -44507,8 +44507,8 @@
       <c r="C34" s="53"/>
       <c r="D34" s="54"/>
       <c r="E34" s="25"/>
-      <c r="F34" s="83"/>
-      <c r="G34" s="84"/>
+      <c r="F34" s="82"/>
+      <c r="G34" s="79"/>
       <c r="H34" s="5"/>
       <c r="I34" s="5"/>
       <c r="J34" s="5"/>
@@ -44522,8 +44522,8 @@
       <c r="C35" s="53"/>
       <c r="D35" s="26"/>
       <c r="E35" s="26"/>
-      <c r="F35" s="67"/>
-      <c r="G35" s="63"/>
+      <c r="F35" s="65"/>
+      <c r="G35" s="67"/>
       <c r="H35" s="5"/>
       <c r="I35" s="5"/>
       <c r="J35" s="5"/>
@@ -44549,7 +44549,7 @@
     <row r="37" spans="1:13" ht="15.75" customHeight="1">
       <c r="A37" s="24"/>
       <c r="B37" s="45"/>
-      <c r="C37" s="85">
+      <c r="C37" s="89">
         <v>10</v>
       </c>
       <c r="D37" s="23"/>
@@ -44569,8 +44569,8 @@
       <c r="C38" s="86"/>
       <c r="D38" s="23"/>
       <c r="E38" s="36"/>
-      <c r="F38" s="79"/>
-      <c r="G38" s="77"/>
+      <c r="F38" s="76"/>
+      <c r="G38" s="83"/>
       <c r="H38" s="5"/>
       <c r="I38" s="5"/>
       <c r="J38" s="5"/>
@@ -44584,8 +44584,8 @@
       <c r="C39" s="53"/>
       <c r="D39" s="23"/>
       <c r="E39" s="57"/>
-      <c r="F39" s="67"/>
-      <c r="G39" s="63"/>
+      <c r="F39" s="65"/>
+      <c r="G39" s="67"/>
       <c r="H39" s="5"/>
       <c r="I39" s="5"/>
       <c r="J39" s="5"/>
@@ -44598,10 +44598,10 @@
       <c r="B40" s="24"/>
       <c r="C40" s="53"/>
       <c r="D40" s="23"/>
-      <c r="E40" s="85">
+      <c r="E40" s="89">
         <v>4</v>
       </c>
-      <c r="F40" s="87"/>
+      <c r="F40" s="90"/>
       <c r="G40" s="88"/>
       <c r="H40" s="5"/>
       <c r="I40" s="5"/>
@@ -44631,8 +44631,8 @@
       <c r="C42" s="53"/>
       <c r="D42" s="55"/>
       <c r="E42" s="59"/>
-      <c r="F42" s="90"/>
-      <c r="G42" s="89"/>
+      <c r="F42" s="91"/>
+      <c r="G42" s="92"/>
       <c r="H42" s="5"/>
       <c r="I42" s="5"/>
       <c r="J42" s="5"/>
@@ -44644,12 +44644,12 @@
       <c r="A43" s="24"/>
       <c r="B43" s="24"/>
       <c r="C43" s="60"/>
-      <c r="D43" s="85">
+      <c r="D43" s="89">
         <v>8</v>
       </c>
       <c r="E43" s="23"/>
-      <c r="F43" s="67"/>
-      <c r="G43" s="63"/>
+      <c r="F43" s="65"/>
+      <c r="G43" s="67"/>
       <c r="H43" s="5"/>
       <c r="I43" s="5"/>
       <c r="J43" s="5"/>
@@ -44663,8 +44663,8 @@
       <c r="C44" s="31"/>
       <c r="D44" s="86"/>
       <c r="E44" s="23"/>
-      <c r="F44" s="78"/>
-      <c r="G44" s="65"/>
+      <c r="F44" s="80"/>
+      <c r="G44" s="63"/>
       <c r="H44" s="5"/>
       <c r="I44" s="5"/>
       <c r="J44" s="5"/>
@@ -44693,8 +44693,8 @@
       <c r="C46" s="31"/>
       <c r="D46" s="61"/>
       <c r="E46" s="23"/>
-      <c r="F46" s="79"/>
-      <c r="G46" s="77"/>
+      <c r="F46" s="76"/>
+      <c r="G46" s="83"/>
       <c r="H46" s="5"/>
       <c r="I46" s="5"/>
       <c r="J46" s="5"/>
@@ -44708,8 +44708,8 @@
       <c r="C47" s="31"/>
       <c r="D47" s="23"/>
       <c r="E47" s="43"/>
-      <c r="F47" s="67"/>
-      <c r="G47" s="63"/>
+      <c r="F47" s="65"/>
+      <c r="G47" s="67"/>
       <c r="H47" s="5"/>
       <c r="I47" s="5"/>
       <c r="J47" s="5"/>
@@ -59134,11 +59134,28 @@
     </row>
   </sheetData>
   <mergeCells count="43">
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="E40:E41"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="G42:G43"/>
+    <mergeCell ref="D43:D44"/>
+    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="F42:F43"/>
+    <mergeCell ref="F46:F47"/>
+    <mergeCell ref="G46:G47"/>
+    <mergeCell ref="F38:F39"/>
+    <mergeCell ref="G38:G39"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="F26:F27"/>
+    <mergeCell ref="G26:G27"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="E28:E29"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F30:F31"/>
+    <mergeCell ref="G30:G31"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="F34:F35"/>
+    <mergeCell ref="G34:G35"/>
     <mergeCell ref="D7:D8"/>
     <mergeCell ref="F8:G8"/>
     <mergeCell ref="D19:D20"/>
@@ -59155,28 +59172,11 @@
     <mergeCell ref="F18:F19"/>
     <mergeCell ref="G18:G19"/>
     <mergeCell ref="F22:F23"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="E28:E29"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F30:F31"/>
-    <mergeCell ref="G30:G31"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="F34:F35"/>
-    <mergeCell ref="G34:G35"/>
-    <mergeCell ref="F46:F47"/>
-    <mergeCell ref="G46:G47"/>
-    <mergeCell ref="F38:F39"/>
-    <mergeCell ref="G38:G39"/>
-    <mergeCell ref="G22:G23"/>
-    <mergeCell ref="F26:F27"/>
-    <mergeCell ref="G26:G27"/>
-    <mergeCell ref="E40:E41"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="G42:G43"/>
-    <mergeCell ref="D43:D44"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="F42:F43"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="G6:G7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>